<commit_message>
Feat: Ajustar regras de distribuição e redistribuição
- Importação distribui apenas por fila e usuários online no horário
- SS respondida existente vira status respondida
- SS respondida nova é atribuída e marcada respondida
- Salvar fila na SS ao importar
- Redistribuição automática por fila e horário
- Filtro por SS/placa na redistribuição
- Redistribuição individual usando seletor
- Status efetivo no modal de redistribuição
</commit_message>
<xml_diff>
--- a/exemplo_importacao.xlsx
+++ b/exemplo_importacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://localiza-my.sharepoint.com/personal/luis_philippe_localiza_com/Documents/Área de Trabalho/Sistema - Pos contato/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="11_26F7C61BAA387D6A2061028C30549827A12CD417" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18923FEB-4DD9-4A0B-BDD5-153285B1ABF2}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="11_26F7C61BAA387D6A2061028C30549827A12CD417" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F6E40E1-ADA2-422B-B21A-22AEAE120EFC}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="171">
   <si>
     <t>ss_data_saida_real</t>
   </si>
@@ -304,9 +304,6 @@
   </si>
   <si>
     <t>Pós Rápidos e Médios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">	Pós Complexo</t>
   </si>
   <si>
     <t>SS00110</t>
@@ -556,6 +553,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="d/m/yy\ h:mm;@"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -593,7 +593,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -936,13 +936,13 @@
   <dimension ref="A1:R28"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="19.25" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.33203125" customWidth="1"/>
     <col min="11" max="11" width="18.4140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -996,7 +996,7 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
-        <v>46082</v>
+        <v>46082.625</v>
       </c>
       <c r="B2" t="s">
         <v>89</v>
@@ -1017,10 +1017,10 @@
         <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J2" t="s">
         <v>22</v>
@@ -1052,7 +1052,7 @@
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
-        <v>46083</v>
+        <v>46083.666666666664</v>
       </c>
       <c r="B3" t="s">
         <v>89</v>
@@ -1073,10 +1073,10 @@
         <v>32</v>
       </c>
       <c r="H3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J3" t="s">
         <v>33</v>
@@ -1108,7 +1108,7 @@
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
-        <v>46084</v>
+        <v>46084.70833321759</v>
       </c>
       <c r="B4" t="s">
         <v>89</v>
@@ -1129,10 +1129,10 @@
         <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J4" t="s">
         <v>43</v>
@@ -1164,7 +1164,7 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
-        <v>46085</v>
+        <v>46085.749999826388</v>
       </c>
       <c r="B5" t="s">
         <v>89</v>
@@ -1185,10 +1185,10 @@
         <v>50</v>
       </c>
       <c r="H5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J5" t="s">
         <v>51</v>
@@ -1220,7 +1220,7 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
-        <v>46086</v>
+        <v>46086.791666435187</v>
       </c>
       <c r="B6" t="s">
         <v>89</v>
@@ -1241,10 +1241,10 @@
         <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J6" t="s">
         <v>22</v>
@@ -1276,7 +1276,7 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
-        <v>46087</v>
+        <v>46087.833333043978</v>
       </c>
       <c r="B7" t="s">
         <v>89</v>
@@ -1297,10 +1297,10 @@
         <v>21</v>
       </c>
       <c r="H7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J7" t="s">
         <v>22</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
-        <v>46088</v>
+        <v>46088.874999652777</v>
       </c>
       <c r="B8" t="s">
         <v>89</v>
@@ -1353,10 +1353,10 @@
         <v>32</v>
       </c>
       <c r="H8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J8" t="s">
         <v>33</v>
@@ -1388,7 +1388,7 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
-        <v>46089</v>
+        <v>46089.916666261575</v>
       </c>
       <c r="B9" t="s">
         <v>89</v>
@@ -1409,10 +1409,10 @@
         <v>42</v>
       </c>
       <c r="H9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J9" t="s">
         <v>43</v>
@@ -1444,7 +1444,7 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
-        <v>46090</v>
+        <v>46090.958332870374</v>
       </c>
       <c r="B10" t="s">
         <v>89</v>
@@ -1465,10 +1465,10 @@
         <v>50</v>
       </c>
       <c r="H10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J10" t="s">
         <v>51</v>
@@ -1500,7 +1500,7 @@
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
-        <v>46091</v>
+        <v>46091.999999479165</v>
       </c>
       <c r="B11" t="s">
         <v>89</v>
@@ -1521,10 +1521,10 @@
         <v>60</v>
       </c>
       <c r="H11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J11" t="s">
         <v>22</v>
@@ -1556,7 +1556,7 @@
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
-        <v>46092</v>
+        <v>46093.041666087964</v>
       </c>
       <c r="B12" t="s">
         <v>89</v>
@@ -1577,10 +1577,10 @@
         <v>21</v>
       </c>
       <c r="H12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J12" t="s">
         <v>22</v>
@@ -1612,7 +1612,7 @@
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
-        <v>46093</v>
+        <v>46094.083332696762</v>
       </c>
       <c r="B13" t="s">
         <v>89</v>
@@ -1633,10 +1633,10 @@
         <v>32</v>
       </c>
       <c r="H13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J13" t="s">
         <v>33</v>
@@ -1668,7 +1668,7 @@
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
-        <v>46094</v>
+        <v>46095.124999305554</v>
       </c>
       <c r="B14" t="s">
         <v>89</v>
@@ -1689,10 +1689,10 @@
         <v>42</v>
       </c>
       <c r="H14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J14" t="s">
         <v>43</v>
@@ -1724,10 +1724,10 @@
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
-        <v>46095</v>
+        <v>46096.166665914352</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
         <v>17</v>
@@ -1745,10 +1745,10 @@
         <v>50</v>
       </c>
       <c r="H15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J15" t="s">
         <v>51</v>
@@ -1780,10 +1780,10 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
-        <v>46096</v>
+        <v>46097.208332523151</v>
       </c>
       <c r="B16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C16" t="s">
         <v>57</v>
@@ -1801,10 +1801,10 @@
         <v>60</v>
       </c>
       <c r="H16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I16" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J16" t="s">
         <v>22</v>
@@ -1836,10 +1836,10 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
-        <v>46097</v>
+        <v>46098.249999131942</v>
       </c>
       <c r="B17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
         <v>17</v>
@@ -1857,10 +1857,10 @@
         <v>21</v>
       </c>
       <c r="H17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J17" t="s">
         <v>22</v>
@@ -1892,10 +1892,10 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
-        <v>46098</v>
+        <v>46099.29166574074</v>
       </c>
       <c r="B18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C18" t="s">
         <v>29</v>
@@ -1913,10 +1913,10 @@
         <v>32</v>
       </c>
       <c r="H18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I18" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J18" t="s">
         <v>33</v>
@@ -1948,10 +1948,10 @@
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
-        <v>46099</v>
+        <v>46100.333332349539</v>
       </c>
       <c r="B19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C19" t="s">
         <v>39</v>
@@ -1969,10 +1969,10 @@
         <v>42</v>
       </c>
       <c r="H19" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I19" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J19" t="s">
         <v>43</v>
@@ -2004,10 +2004,10 @@
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
-        <v>46100</v>
+        <v>46101.37499895833</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
         <v>17</v>
@@ -2025,10 +2025,10 @@
         <v>50</v>
       </c>
       <c r="H20" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I20" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J20" t="s">
         <v>51</v>
@@ -2060,10 +2060,10 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
-        <v>46101</v>
+        <v>46102.416665567129</v>
       </c>
       <c r="B21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C21" t="s">
         <v>57</v>
@@ -2081,10 +2081,10 @@
         <v>60</v>
       </c>
       <c r="H21" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I21" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J21" t="s">
         <v>22</v>
@@ -2116,10 +2116,10 @@
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
-        <v>46102</v>
+        <v>46103.458332175927</v>
       </c>
       <c r="B22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C22" t="s">
         <v>17</v>
@@ -2137,10 +2137,10 @@
         <v>21</v>
       </c>
       <c r="H22" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I22" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J22" t="s">
         <v>22</v>
@@ -2172,10 +2172,10 @@
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
-        <v>46103</v>
+        <v>46104.499998784719</v>
       </c>
       <c r="B23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C23" t="s">
         <v>29</v>
@@ -2193,10 +2193,10 @@
         <v>32</v>
       </c>
       <c r="H23" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I23" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J23" t="s">
         <v>33</v>
@@ -2228,10 +2228,10 @@
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
-        <v>46104</v>
+        <v>46105.541665393517</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C24" t="s">
         <v>39</v>
@@ -2249,10 +2249,10 @@
         <v>42</v>
       </c>
       <c r="H24" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I24" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J24" t="s">
         <v>43</v>
@@ -2284,10 +2284,10 @@
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
-        <v>46105</v>
+        <v>46106.583332002316</v>
       </c>
       <c r="B25" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C25" t="s">
         <v>17</v>
@@ -2305,10 +2305,10 @@
         <v>50</v>
       </c>
       <c r="H25" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I25" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J25" t="s">
         <v>51</v>
@@ -2340,10 +2340,10 @@
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
-        <v>46106</v>
+        <v>46107.624998611114</v>
       </c>
       <c r="B26" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C26" t="s">
         <v>57</v>
@@ -2361,10 +2361,10 @@
         <v>60</v>
       </c>
       <c r="H26" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I26" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J26" t="s">
         <v>22</v>
@@ -2396,10 +2396,10 @@
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
-        <v>46107</v>
+        <v>46108.666665219906</v>
       </c>
       <c r="B27" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C27" t="s">
         <v>17</v>
@@ -2417,10 +2417,10 @@
         <v>21</v>
       </c>
       <c r="H27" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I27" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J27" t="s">
         <v>22</v>
@@ -2452,10 +2452,10 @@
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
-        <v>46108</v>
+        <v>46109.708331828704</v>
       </c>
       <c r="B28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C28" t="s">
         <v>29</v>
@@ -2473,10 +2473,10 @@
         <v>32</v>
       </c>
       <c r="H28" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I28" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J28" t="s">
         <v>33</v>
@@ -2533,7 +2533,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B2" t="str">
         <f>A2&amp;3</f>
@@ -2542,7 +2542,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" ref="B3:B28" si="0">A3&amp;3</f>
@@ -2551,7 +2551,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
@@ -2560,7 +2560,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
@@ -2569,7 +2569,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
@@ -2578,7 +2578,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
@@ -2587,7 +2587,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
@@ -2596,7 +2596,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
@@ -2605,7 +2605,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -2614,7 +2614,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
@@ -2623,7 +2623,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
@@ -2632,7 +2632,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
@@ -2650,7 +2650,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
@@ -2659,7 +2659,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
@@ -2668,7 +2668,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
@@ -2677,7 +2677,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
@@ -2686,7 +2686,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
@@ -2695,7 +2695,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
@@ -2704,7 +2704,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
@@ -2713,7 +2713,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
@@ -2722,7 +2722,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
@@ -2731,7 +2731,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
@@ -2740,7 +2740,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
@@ -2749,7 +2749,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
@@ -2758,7 +2758,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
@@ -2767,7 +2767,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>

</xml_diff>